<commit_message>
New and Updated System
</commit_message>
<xml_diff>
--- a/frontend/public/templates/student-import-template.xlsx
+++ b/frontend/public/templates/student-import-template.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="1" r:id="Rc42917f827864768"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="1" r:id="R607f6dc0b3a04136"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grades" sheetId="2" r:id="R037e465b26814f21"/>
   </sheets>
 </workbook>
 </file>
@@ -13,9 +14,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="200" formatCode="0"/>
     <numFmt numFmtId="201" formatCode="@"/>
+    <numFmt numFmtId="202" formatCode="0.##"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -45,12 +47,22 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF168CC8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFBEB"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -69,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -95,10 +107,29 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="202" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FFBE123C"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF1F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -386,16 +417,25 @@
       <c r="A10" s="7"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
+      <c r="E10" s="9" t="str">
+        <v>Optional: use the Grades worksheet for existing term grades by subject.</v>
+      </c>
     </row>
     <row r="11" ht="23" customHeight="1">
       <c r="A11" s="7"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
+      <c r="E11" s="9" t="str">
+        <v>Repeat the same student details in Grades and enter the selected subject name.</v>
+      </c>
     </row>
     <row r="12" ht="23" customHeight="1">
       <c r="A12" s="7"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
+      <c r="E12" s="9" t="str">
+        <v>Imports use the active school year. Saved grades are preserved.</v>
+      </c>
     </row>
     <row r="13" ht="23" customHeight="1">
       <c r="A13" s="7"/>
@@ -5350,4 +5390,538 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="21" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="35" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="3" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="105" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="23" customHeight="1">
+      <c r="A1" s="13" t="str">
+        <v>Grade Level</v>
+      </c>
+      <c r="B1" s="13" t="str">
+        <v>Section</v>
+      </c>
+      <c r="C1" s="13" t="str">
+        <v>Student Name</v>
+      </c>
+      <c r="D1" s="13" t="str">
+        <v>Subject</v>
+      </c>
+      <c r="E1" s="13" t="str">
+        <v>Term 1 Grade</v>
+      </c>
+      <c r="F1" s="13" t="str">
+        <v>Term 2 Grade</v>
+      </c>
+      <c r="G1" s="13" t="str">
+        <v>Term 3 Grade</v>
+      </c>
+      <c r="I1" s="10" t="str">
+        <v>Import existing grades (optional)</v>
+      </c>
+    </row>
+    <row r="2" ht="23" customHeight="1">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="I2" s="9" t="str">
+        <v>Use one row per student and subject, starting in row 2.</v>
+      </c>
+    </row>
+    <row r="3" ht="23" customHeight="1">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="I3" s="9" t="str">
+        <v>Copy Grade Level, Section and Student Name from the Students worksheet.</v>
+      </c>
+    </row>
+    <row r="4" ht="23" customHeight="1">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="I4" s="9" t="str">
+        <v>Subject: enter the exact name of a subject selected on the upload screen.</v>
+      </c>
+    </row>
+    <row r="5" ht="23" customHeight="1">
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="I5" s="9" t="str">
+        <v>Enter existing final Term 1, Term 2 and Term 3 grades from 0 to 100.</v>
+      </c>
+    </row>
+    <row r="6" ht="23" customHeight="1">
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="I6" s="9" t="str">
+        <v>Leave unavailable term grades blank. Zero is a real grade, not a blank.</v>
+      </c>
+    </row>
+    <row r="7" ht="23" customHeight="1">
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="I7" s="9" t="str">
+        <v>Use plain values, with up to two decimal places. Do not use formulas.</v>
+      </c>
+    </row>
+    <row r="8" ht="23" customHeight="1">
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="I8" s="9" t="str">
+        <v>Existing students must already be enrolled. Saved imported grades are preserved.</v>
+      </c>
+    </row>
+    <row r="9" ht="23" customHeight="1">
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="I9" s="9" t="str">
+        <v>Complete assessment-based grades take precedence over imported grades.</v>
+      </c>
+    </row>
+    <row r="10" ht="23" customHeight="1">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="I10" s="9" t="str">
+        <v>Use the active school year. Up to 10,000 grade rows per file.</v>
+      </c>
+    </row>
+    <row r="11" ht="23" customHeight="1">
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+    </row>
+    <row r="12" ht="23" customHeight="1">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+    </row>
+    <row r="13" ht="23" customHeight="1">
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+    </row>
+    <row r="14" ht="23" customHeight="1">
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+    </row>
+    <row r="15" ht="23" customHeight="1">
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+    </row>
+    <row r="16" ht="23" customHeight="1">
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+    </row>
+    <row r="17" ht="23" customHeight="1">
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+    </row>
+    <row r="18" ht="23" customHeight="1">
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+    </row>
+    <row r="19" ht="23" customHeight="1">
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+    </row>
+    <row r="20" ht="23" customHeight="1">
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+    </row>
+    <row r="21" ht="23" customHeight="1">
+      <c r="A21" s="14"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+    </row>
+    <row r="22" ht="23" customHeight="1">
+      <c r="A22" s="14"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+    </row>
+    <row r="23" ht="23" customHeight="1">
+      <c r="A23" s="14"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+    </row>
+    <row r="24" ht="23" customHeight="1">
+      <c r="A24" s="14"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+    </row>
+    <row r="25" ht="23" customHeight="1">
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+    </row>
+    <row r="26" ht="23" customHeight="1">
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+    </row>
+    <row r="27" ht="23" customHeight="1">
+      <c r="A27" s="14"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+    </row>
+    <row r="28" ht="23" customHeight="1">
+      <c r="A28" s="14"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+    </row>
+    <row r="29" ht="23" customHeight="1">
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+    </row>
+    <row r="30" ht="23" customHeight="1">
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+    </row>
+    <row r="31" ht="23" customHeight="1">
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+    </row>
+    <row r="32" ht="23" customHeight="1">
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+    </row>
+    <row r="33" ht="23" customHeight="1">
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+    </row>
+    <row r="34" ht="23" customHeight="1">
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+    </row>
+    <row r="35" ht="23" customHeight="1">
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+    </row>
+    <row r="36" ht="23" customHeight="1">
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+    </row>
+    <row r="37" ht="23" customHeight="1">
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+    </row>
+    <row r="38" ht="23" customHeight="1">
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+    </row>
+    <row r="39" ht="23" customHeight="1">
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+    </row>
+    <row r="40" ht="23" customHeight="1">
+      <c r="A40" s="14"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+    </row>
+    <row r="41" ht="23" customHeight="1">
+      <c r="A41" s="14"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+    </row>
+    <row r="42" ht="23" customHeight="1">
+      <c r="A42" s="14"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+    </row>
+    <row r="43" ht="23" customHeight="1">
+      <c r="A43" s="14"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+    </row>
+    <row r="44" ht="23" customHeight="1">
+      <c r="A44" s="14"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+    </row>
+    <row r="45" ht="23" customHeight="1">
+      <c r="A45" s="14"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="15"/>
+    </row>
+    <row r="46" ht="23" customHeight="1">
+      <c r="A46" s="14"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+    </row>
+    <row r="47" ht="23" customHeight="1">
+      <c r="A47" s="14"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+    </row>
+    <row r="48" ht="23" customHeight="1">
+      <c r="A48" s="14"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+    </row>
+    <row r="49" ht="23" customHeight="1">
+      <c r="A49" s="14"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="15"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="15"/>
+    </row>
+    <row r="50" ht="23" customHeight="1">
+      <c r="A50" s="14"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="14"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="15"/>
+    </row>
+    <row r="51" ht="23" customHeight="1">
+      <c r="A51" s="14"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:G1001">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND(E2&lt;&gt;"",IF(ISNUMBER(E2),OR(E2&lt;0,E2&gt;100,ROUND(E2,2)&lt;&gt;E2),TRUE))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="whole" errorStyle="stop" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Grade level" error="Enter a positive whole-number grade level." sqref="A2:A10001">
+      <formula1>1</formula1>
+      <formula2>99</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>